<commit_message>
Ducmentacion de Indicadores - Menage 1
</commit_message>
<xml_diff>
--- a/Liste_parameters.xlsx
+++ b/Liste_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thesis\03-Code_Storage\02-Altintlas_Nessy2m_Storage\Chatter-Criteria\CAMP10_Chatter_detection_Methodes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D43833-2739-4353-B660-2295AA16174A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27AAB29-3A0A-46BF-9C51-CEC380A0B233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="29829" windowHeight="18000" activeTab="1" xr2:uid="{CFC0A26A-5BC2-4561-8ED4-277EBA2C2982}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="88">
   <si>
     <t xml:space="preserve">Optional </t>
   </si>
@@ -166,6 +166,141 @@
   </si>
   <si>
     <t>dt_rms</t>
+  </si>
+  <si>
+    <t>_maxent_sprt_pipeline</t>
+  </si>
+  <si>
+    <t>rpm</t>
+  </si>
+  <si>
+    <t>ratio_sampling</t>
+  </si>
+  <si>
+    <t>N_seg</t>
+  </si>
+  <si>
+    <t>t_stable_total</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>reset_on_H0</t>
+  </si>
+  <si>
+    <t>cut_start_time</t>
+  </si>
+  <si>
+    <t>cut_end_time</t>
+  </si>
+  <si>
+    <t>sample_opr</t>
+  </si>
+  <si>
+    <t>fr</t>
+  </si>
+  <si>
+    <t>np.ndarray</t>
+  </si>
+  <si>
+    <t>MaxEntSPRTConfig</t>
+  </si>
+  <si>
+    <t>MaxEntSPRTDetector</t>
+  </si>
+  <si>
+    <t>models</t>
+  </si>
+  <si>
+    <t>config</t>
+  </si>
+  <si>
+    <t>estimator</t>
+  </si>
+  <si>
+    <t>H_free</t>
+  </si>
+  <si>
+    <t>Atributo</t>
+  </si>
+  <si>
+    <t>H_chat</t>
+  </si>
+  <si>
+    <t>t_mid_free</t>
+  </si>
+  <si>
+    <t>t_mid_chat</t>
+  </si>
+  <si>
+    <t>MaxEntModels | None</t>
+  </si>
+  <si>
+    <t>EntropyEstimator</t>
+  </si>
+  <si>
+    <t>np.ndarray | None</t>
+  </si>
+  <si>
+    <t>fit_offline_from_opr</t>
+  </si>
+  <si>
+    <t>opr_free</t>
+  </si>
+  <si>
+    <t>opr_t_free</t>
+  </si>
+  <si>
+    <t>opr_chat</t>
+  </si>
+  <si>
+    <t>opr_t_chat</t>
+  </si>
+  <si>
+    <t>offline_train_maxent_sprt</t>
+  </si>
+  <si>
+    <t>segment_opr</t>
+  </si>
+  <si>
+    <t>opr</t>
+  </si>
+  <si>
+    <t>opr_t</t>
+  </si>
+  <si>
+    <t>entropy_from_segments</t>
+  </si>
+  <si>
+    <t>segments</t>
+  </si>
+  <si>
+    <t>Sequence[np.ndarray]</t>
+  </si>
+  <si>
+    <t>entropy_from_segment</t>
+  </si>
+  <si>
+    <t>seg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parametros </t>
+  </si>
+  <si>
+    <t>Parametros</t>
+  </si>
+  <si>
+    <t>t_chatter_total</t>
+  </si>
+  <si>
+    <t>signal_chatter</t>
+  </si>
+  <si>
+    <t>signal_stable</t>
   </si>
 </sst>
 </file>
@@ -537,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A46004D4-5D69-4C97-B1BF-25B5DB9CC174}">
-  <dimension ref="B1:L31"/>
+  <dimension ref="B1:L33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1120,6 +1255,9 @@
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B23" t="s">
+        <v>83</v>
+      </c>
       <c r="H23" t="s">
         <v>5</v>
       </c>
@@ -1137,6 +1275,9 @@
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
       <c r="H24" t="s">
         <v>6</v>
       </c>
@@ -1154,6 +1295,9 @@
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
       <c r="H25" t="s">
         <v>10</v>
       </c>
@@ -1171,6 +1315,9 @@
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B26" t="s">
+        <v>23</v>
+      </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
@@ -1188,6 +1335,9 @@
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B27" t="s">
+        <v>40</v>
+      </c>
       <c r="H27" t="s">
         <v>12</v>
       </c>
@@ -1205,6 +1355,9 @@
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
       <c r="H28" t="s">
         <v>13</v>
       </c>
@@ -1222,6 +1375,9 @@
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B29" t="s">
+        <v>10</v>
+      </c>
       <c r="H29" t="s">
         <v>14</v>
       </c>
@@ -1239,6 +1395,9 @@
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B30" t="s">
+        <v>11</v>
+      </c>
       <c r="H30" t="s">
         <v>42</v>
       </c>
@@ -1256,6 +1415,9 @@
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
       <c r="H31" t="s">
         <v>15</v>
       </c>
@@ -1270,11 +1432,31 @@
       </c>
       <c r="L31" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.4">
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="B33" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:E1048576">
     <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1293,8 +1475,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="I4:J6">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I1:K1">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1313,8 +1505,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:J6">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="K3">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1333,8 +1525,946 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K3">
-    <cfRule type="colorScale" priority="2">
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960EC801-918C-4D31-8889-BA2AA7AE028E}">
+  <dimension ref="B1:S39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="25.765625" customWidth="1"/>
+    <col min="5" max="5" width="13.3828125" customWidth="1"/>
+    <col min="6" max="6" width="13.4609375" customWidth="1"/>
+    <col min="7" max="7" width="3.3046875" customWidth="1"/>
+    <col min="8" max="8" width="19.3046875" customWidth="1"/>
+    <col min="9" max="9" width="14.3046875" customWidth="1"/>
+    <col min="12" max="12" width="14.69140625" customWidth="1"/>
+    <col min="13" max="13" width="23.15234375" customWidth="1"/>
+    <col min="14" max="14" width="4" customWidth="1"/>
+    <col min="15" max="15" width="21.84375" customWidth="1"/>
+    <col min="19" max="19" width="15.4609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" t="s">
+        <v>39</v>
+      </c>
+      <c r="S1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P3" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" t="s">
+        <v>50</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" t="s">
+        <v>57</v>
+      </c>
+      <c r="O14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" t="s">
+        <v>58</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>66</v>
+      </c>
+      <c r="O15" t="s">
+        <v>70</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="H16" t="s">
+        <v>59</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>56</v>
+      </c>
+      <c r="O16" t="s">
+        <v>71</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="H17" t="s">
+        <v>60</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17" t="s">
+        <v>67</v>
+      </c>
+      <c r="O17" t="s">
+        <v>72</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>1</v>
+      </c>
+      <c r="S17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" t="s">
+        <v>61</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18" t="s">
+        <v>68</v>
+      </c>
+      <c r="O18" t="s">
+        <v>73</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>1</v>
+      </c>
+      <c r="S18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" t="s">
+        <v>63</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
+        <v>68</v>
+      </c>
+      <c r="O19" t="s">
+        <v>46</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" t="s">
+        <v>64</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>68</v>
+      </c>
+      <c r="O20" t="s">
+        <v>60</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+      <c r="S20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="O22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+      <c r="O23" t="s">
+        <v>70</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
+      <c r="S23" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="O24" t="s">
+        <v>71</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
+      <c r="S24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B25" t="s">
+        <v>47</v>
+      </c>
+      <c r="O25" t="s">
+        <v>72</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>1</v>
+      </c>
+      <c r="S25" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B26" t="s">
+        <v>85</v>
+      </c>
+      <c r="O26" t="s">
+        <v>73</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>1</v>
+      </c>
+      <c r="S26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+      <c r="O27" t="s">
+        <v>46</v>
+      </c>
+      <c r="P27">
+        <v>0</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B29" t="s">
+        <v>48</v>
+      </c>
+      <c r="O29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="O30" t="s">
+        <v>76</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>1</v>
+      </c>
+      <c r="S30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="B31" t="s">
+        <v>50</v>
+      </c>
+      <c r="O31" t="s">
+        <v>77</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>1</v>
+      </c>
+      <c r="S31" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="O32" t="s">
+        <v>46</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="15:19" x14ac:dyDescent="0.4">
+      <c r="O34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="15:19" x14ac:dyDescent="0.4">
+      <c r="O35" t="s">
+        <v>79</v>
+      </c>
+      <c r="P35">
+        <v>0</v>
+      </c>
+      <c r="Q35">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>1</v>
+      </c>
+      <c r="S35" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="15:19" x14ac:dyDescent="0.4">
+      <c r="O36" t="s">
+        <v>60</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="Q36">
+        <v>0</v>
+      </c>
+      <c r="R36">
+        <v>1</v>
+      </c>
+      <c r="S36" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="38" spans="15:19" x14ac:dyDescent="0.4">
+      <c r="O38" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="15:19" x14ac:dyDescent="0.4">
+      <c r="O39" t="s">
+        <v>82</v>
+      </c>
+      <c r="P39">
+        <v>0</v>
+      </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>1</v>
+      </c>
+      <c r="S39" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C1:E3 C10:E1048576 C7:E8 P1:R20 P22:R1048576">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1343,8 +2473,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:K1">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="J3">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1353,85 +2483,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960EC801-918C-4D31-8889-BA2AA7AE028E}">
-  <dimension ref="B1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="25.765625" customWidth="1"/>
-    <col min="5" max="5" width="13.3828125" customWidth="1"/>
-    <col min="7" max="7" width="3.3046875" customWidth="1"/>
-    <col min="8" max="8" width="19.3046875" customWidth="1"/>
-    <col min="11" max="11" width="14.69140625" customWidth="1"/>
-    <col min="12" max="12" width="23.15234375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.4">
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.4">
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" t="s">
-        <v>1</v>
-      </c>
-      <c r="I3" t="s">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="C1:E1048576">
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="J2:K2 J8:K9 J13:K1048576">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -1440,7 +2493,117 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:J2 I7:J1048576">
+  <conditionalFormatting sqref="J4:K7">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:L1">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L4:L9 L2 L13:L1048576">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:E9">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:E5">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:E6">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J10:L12">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4:I1048576 I1:I2">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:Q2">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1450,17 +2613,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFFF0000"/>
-        <color theme="9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3">
+  <conditionalFormatting sqref="Q3">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1470,17 +2623,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:J6">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFFF0000"/>
-        <color theme="9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4:K1048576 K2">
+  <conditionalFormatting sqref="R3">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1490,18 +2633,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K3">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFFF0000"/>
-        <color theme="9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I1:K1">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="R2">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>

</xml_diff>

<commit_message>
Posible Error en MaxEnt en la varaible ratio_samplig (posible param optionel)
</commit_message>
<xml_diff>
--- a/Liste_parameters.xlsx
+++ b/Liste_parameters.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Thesis\03-Code_Storage\02-Altintlas_Nessy2m_Storage\Chatter-Criteria\CAMP10_Chatter_detection_Methodes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27AAB29-3A0A-46BF-9C51-CEC380A0B233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB4D033-7269-456D-AD14-5E3A48D803FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="29829" windowHeight="18000" activeTab="1" xr2:uid="{CFC0A26A-5BC2-4561-8ED4-277EBA2C2982}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="29829" windowHeight="18000" xr2:uid="{CFC0A26A-5BC2-4561-8ED4-277EBA2C2982}"/>
   </bookViews>
   <sheets>
     <sheet name="RMS" sheetId="1" r:id="rId1"/>
     <sheet name="MaxEnt_SPRT" sheetId="2" r:id="rId2"/>
+    <sheet name="SST_SVD" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="100">
   <si>
     <t xml:space="preserve">Optional </t>
   </si>
@@ -198,6 +199,9 @@
     <t>cut_end_time</t>
   </si>
   <si>
+    <t>SignalData</t>
+  </si>
+  <si>
     <t>sample_opr</t>
   </si>
   <si>
@@ -301,6 +305,39 @@
   </si>
   <si>
     <t>signal_stable</t>
+  </si>
+  <si>
+    <t>sst_svd_pipeline</t>
+  </si>
+  <si>
+    <t>n_fft_power</t>
+  </si>
+  <si>
+    <t>win_length_ms</t>
+  </si>
+  <si>
+    <t>hop_ms</t>
+  </si>
+  <si>
+    <t>Ai_length</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>sigma</t>
+  </si>
+  <si>
+    <t>frac_stable</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>fallback_mad</t>
+  </si>
+  <si>
+    <t>str</t>
   </si>
 </sst>
 </file>
@@ -1256,7 +1293,7 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.4">
       <c r="B23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H23" t="s">
         <v>5</v>
@@ -1562,7 +1599,7 @@
         <v>2</v>
       </c>
       <c r="I1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1597,7 +1634,7 @@
         <v>43</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.4">
@@ -1676,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="2:19" x14ac:dyDescent="0.4">
@@ -1711,7 +1748,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.4">
@@ -1766,7 +1803,7 @@
         <v>18</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I7" t="s">
         <v>38</v>
@@ -1818,7 +1855,7 @@
         <v>18</v>
       </c>
       <c r="H9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.4">
@@ -1960,10 +1997,10 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.4">
@@ -1983,7 +2020,7 @@
         <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -1998,10 +2035,10 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -2013,12 +2050,12 @@
         <v>1</v>
       </c>
       <c r="S15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.4">
       <c r="H16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -2033,27 +2070,27 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
+        <v>57</v>
+      </c>
+      <c r="O16" t="s">
+        <v>72</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16" t="s">
         <v>56</v>
-      </c>
-      <c r="O16" t="s">
-        <v>71</v>
-      </c>
-      <c r="P16">
-        <v>0</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>1</v>
-      </c>
-      <c r="S16" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="17" spans="2:19" x14ac:dyDescent="0.4">
       <c r="H17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I17">
         <v>1</v>
@@ -2068,10 +2105,10 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P17">
         <v>0</v>
@@ -2083,15 +2120,15 @@
         <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="2:19" x14ac:dyDescent="0.4">
       <c r="B18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I18">
         <v>1</v>
@@ -2106,10 +2143,10 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P18">
         <v>0</v>
@@ -2121,7 +2158,7 @@
         <v>1</v>
       </c>
       <c r="S18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="2:19" x14ac:dyDescent="0.4">
@@ -2129,7 +2166,7 @@
         <v>21</v>
       </c>
       <c r="H19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I19">
         <v>1</v>
@@ -2144,7 +2181,7 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O19" t="s">
         <v>46</v>
@@ -2167,7 +2204,7 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I20">
         <v>1</v>
@@ -2182,22 +2219,22 @@
         <v>1</v>
       </c>
       <c r="M20" t="s">
+        <v>69</v>
+      </c>
+      <c r="O20" t="s">
+        <v>61</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+      <c r="S20" t="s">
         <v>68</v>
-      </c>
-      <c r="O20" t="s">
-        <v>60</v>
-      </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
-        <v>0</v>
-      </c>
-      <c r="R20">
-        <v>1</v>
-      </c>
-      <c r="S20" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="21" spans="2:19" x14ac:dyDescent="0.4">
@@ -2205,7 +2242,7 @@
         <v>23</v>
       </c>
       <c r="H21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -2220,7 +2257,7 @@
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="2:19" x14ac:dyDescent="0.4">
@@ -2228,7 +2265,7 @@
         <v>44</v>
       </c>
       <c r="O22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="2:19" x14ac:dyDescent="0.4">
@@ -2236,7 +2273,7 @@
         <v>45</v>
       </c>
       <c r="O23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="P23">
         <v>0</v>
@@ -2248,7 +2285,7 @@
         <v>1</v>
       </c>
       <c r="S23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="2:19" x14ac:dyDescent="0.4">
@@ -2256,7 +2293,7 @@
         <v>46</v>
       </c>
       <c r="O24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -2268,7 +2305,7 @@
         <v>1</v>
       </c>
       <c r="S24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="2:19" x14ac:dyDescent="0.4">
@@ -2276,7 +2313,7 @@
         <v>47</v>
       </c>
       <c r="O25" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P25">
         <v>0</v>
@@ -2288,15 +2325,15 @@
         <v>1</v>
       </c>
       <c r="S25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="2:19" x14ac:dyDescent="0.4">
       <c r="B26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P26">
         <v>0</v>
@@ -2308,12 +2345,12 @@
         <v>1</v>
       </c>
       <c r="S26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="2:19" x14ac:dyDescent="0.4">
       <c r="B27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O27" t="s">
         <v>46</v>
@@ -2333,7 +2370,7 @@
     </row>
     <row r="28" spans="2:19" x14ac:dyDescent="0.4">
       <c r="B28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="2:19" x14ac:dyDescent="0.4">
@@ -2341,7 +2378,7 @@
         <v>48</v>
       </c>
       <c r="O29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="2:19" x14ac:dyDescent="0.4">
@@ -2349,7 +2386,7 @@
         <v>49</v>
       </c>
       <c r="O30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P30">
         <v>0</v>
@@ -2361,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="S30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="2:19" x14ac:dyDescent="0.4">
@@ -2369,7 +2406,7 @@
         <v>50</v>
       </c>
       <c r="O31" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P31">
         <v>0</v>
@@ -2381,7 +2418,7 @@
         <v>1</v>
       </c>
       <c r="S31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="2:19" x14ac:dyDescent="0.4">
@@ -2403,12 +2440,12 @@
     </row>
     <row r="34" spans="15:19" x14ac:dyDescent="0.4">
       <c r="O34" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="15:19" x14ac:dyDescent="0.4">
       <c r="O35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -2420,12 +2457,12 @@
         <v>1</v>
       </c>
       <c r="S35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="15:19" x14ac:dyDescent="0.4">
       <c r="O36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P36">
         <v>0</v>
@@ -2437,17 +2474,17 @@
         <v>1</v>
       </c>
       <c r="S36" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="15:19" x14ac:dyDescent="0.4">
       <c r="O38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="15:19" x14ac:dyDescent="0.4">
       <c r="O39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P39">
         <v>0</v>
@@ -2459,7 +2496,7 @@
         <v>1</v>
       </c>
       <c r="S39" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2645,4 +2682,267 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088DF921-A397-4A43-B2DE-2A6BC625FE95}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="23.15234375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B1:D1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFF0000"/>
+        <color theme="9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>